<commit_message>
Plot polish: green dashed prediction, wider multi-row panels, CMS label, thinner
- plot_surface_vs_data: prediction drawn as a dashed green line; saved as
  param_pred_<production> by run.py; legend added.
- plot_QV and plot_param_pred: panels wrapped over up to 3 columns / multiple rows
  with wider pads (460x400), so the x-axis reads larger.
- "CMS ETL Preliminary" top-left on every figure (first panel for multi-pad).
- Thinner markers/lines across the plots (fit/law/charge/bias widths reduced,
  marker sizes down); QV: drop the red auto-drawn fit curve, keep only the azure.

FBK-LF sheet already present in the workbook -> its _FBKLF files are produced
automatically by the per-sheet pipeline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parametrization_data.xlsx
+++ b/parametrization_data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardolanteri/Desktop/Parametrization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6ED52CB-5FEC-7941-A5AE-524EA9B19CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA24018-27EA-6B47-BA82-16323926586C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
   </bookViews>
   <sheets>
     <sheet name="HPK" sheetId="1" r:id="rId1"/>
+    <sheet name="FBK-LF" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="242">
   <si>
     <t>V</t>
   </si>
@@ -212,9 +213,6 @@
     <t>12.5</t>
   </si>
   <si>
-    <t>HPK2 W13-3 4e14</t>
-  </si>
-  <si>
     <t>38.5</t>
   </si>
   <si>
@@ -227,9 +225,6 @@
     <t>33.5</t>
   </si>
   <si>
-    <t xml:space="preserve">HPK2 W4-25 8e14 </t>
-  </si>
-  <si>
     <t>2.42</t>
   </si>
   <si>
@@ -272,9 +267,6 @@
     <t>36.50</t>
   </si>
   <si>
-    <t>HPK6 S4-B — 1e15</t>
-  </si>
-  <si>
     <t>70.90</t>
   </si>
   <si>
@@ -314,9 +306,6 @@
     <t>35.27</t>
   </si>
   <si>
-    <t>HPK6 S5-A — 1e15</t>
-  </si>
-  <si>
     <t>0.71</t>
   </si>
   <si>
@@ -359,9 +348,6 @@
     <t>76.44</t>
   </si>
   <si>
-    <t>HPK6 S5-B — 1.5e15</t>
-  </si>
-  <si>
     <t>1.19</t>
   </si>
   <si>
@@ -417,6 +403,369 @@
   </si>
   <si>
     <t>29.1</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>69.0</t>
+  </si>
+  <si>
+    <t>8.8</t>
+  </si>
+  <si>
+    <t>61.2</t>
+  </si>
+  <si>
+    <t>9.6</t>
+  </si>
+  <si>
+    <t>55.7</t>
+  </si>
+  <si>
+    <t>11.2</t>
+  </si>
+  <si>
+    <t>52.1</t>
+  </si>
+  <si>
+    <t>12.9</t>
+  </si>
+  <si>
+    <t>44.2</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>42.3</t>
+  </si>
+  <si>
+    <t>17.2</t>
+  </si>
+  <si>
+    <t>39.9</t>
+  </si>
+  <si>
+    <t>20.4</t>
+  </si>
+  <si>
+    <t>35.3</t>
+  </si>
+  <si>
+    <t>24.9</t>
+  </si>
+  <si>
+    <t>30.6</t>
+  </si>
+  <si>
+    <t>29.2</t>
+  </si>
+  <si>
+    <t>FBK-LF W16-S13</t>
+  </si>
+  <si>
+    <t>FBK-LF W16-S52</t>
+  </si>
+  <si>
+    <t>7.90</t>
+  </si>
+  <si>
+    <t>68.81</t>
+  </si>
+  <si>
+    <t>8.87</t>
+  </si>
+  <si>
+    <t>60.36</t>
+  </si>
+  <si>
+    <t>9.72</t>
+  </si>
+  <si>
+    <t>55.05</t>
+  </si>
+  <si>
+    <t>11.22</t>
+  </si>
+  <si>
+    <t>51.79</t>
+  </si>
+  <si>
+    <t>12.88</t>
+  </si>
+  <si>
+    <t>46.45</t>
+  </si>
+  <si>
+    <t>14.96</t>
+  </si>
+  <si>
+    <t>45.93</t>
+  </si>
+  <si>
+    <t>17.29</t>
+  </si>
+  <si>
+    <t>39.86</t>
+  </si>
+  <si>
+    <t>20.61</t>
+  </si>
+  <si>
+    <t>37.18</t>
+  </si>
+  <si>
+    <t>25.08</t>
+  </si>
+  <si>
+    <t>36.26</t>
+  </si>
+  <si>
+    <t>31.01</t>
+  </si>
+  <si>
+    <t>31.34</t>
+  </si>
+  <si>
+    <t>2.61</t>
+  </si>
+  <si>
+    <t>77.67</t>
+  </si>
+  <si>
+    <t>3.52</t>
+  </si>
+  <si>
+    <t>67.36</t>
+  </si>
+  <si>
+    <t>5.15</t>
+  </si>
+  <si>
+    <t>55.78</t>
+  </si>
+  <si>
+    <t>7.84</t>
+  </si>
+  <si>
+    <t>45.92</t>
+  </si>
+  <si>
+    <t>12.84</t>
+  </si>
+  <si>
+    <t>35.75</t>
+  </si>
+  <si>
+    <t>16.12</t>
+  </si>
+  <si>
+    <t>32.77</t>
+  </si>
+  <si>
+    <t>20.18</t>
+  </si>
+  <si>
+    <t>31.57</t>
+  </si>
+  <si>
+    <t>24.60</t>
+  </si>
+  <si>
+    <t>31.52</t>
+  </si>
+  <si>
+    <t>28.54</t>
+  </si>
+  <si>
+    <t>30.85</t>
+  </si>
+  <si>
+    <t>HPK2 W13-3 - 4e14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HPK2 W4-25 - 8e14 </t>
+  </si>
+  <si>
+    <t>HPK6 S4-B - 1e15</t>
+  </si>
+  <si>
+    <t>HPK6 S5-A - 1e15</t>
+  </si>
+  <si>
+    <t>HPK6 S5-B - 1.5e15</t>
+  </si>
+  <si>
+    <t>2.85</t>
+  </si>
+  <si>
+    <t>76.96</t>
+  </si>
+  <si>
+    <t>4.18</t>
+  </si>
+  <si>
+    <t>62.00</t>
+  </si>
+  <si>
+    <t>5.82</t>
+  </si>
+  <si>
+    <t>50.75</t>
+  </si>
+  <si>
+    <t>8.51</t>
+  </si>
+  <si>
+    <t>42.86</t>
+  </si>
+  <si>
+    <t>13.18</t>
+  </si>
+  <si>
+    <t>35.36</t>
+  </si>
+  <si>
+    <t>16.05</t>
+  </si>
+  <si>
+    <t>32.94</t>
+  </si>
+  <si>
+    <t>20.06</t>
+  </si>
+  <si>
+    <t>32.72</t>
+  </si>
+  <si>
+    <t>24.12</t>
+  </si>
+  <si>
+    <t>31.89</t>
+  </si>
+  <si>
+    <t>29.36</t>
+  </si>
+  <si>
+    <t>2.08</t>
+  </si>
+  <si>
+    <t>86.08</t>
+  </si>
+  <si>
+    <t>2.51</t>
+  </si>
+  <si>
+    <t>70.20</t>
+  </si>
+  <si>
+    <t>3.18</t>
+  </si>
+  <si>
+    <t>63.47</t>
+  </si>
+  <si>
+    <t>4.10</t>
+  </si>
+  <si>
+    <t>47.84</t>
+  </si>
+  <si>
+    <t>5.22</t>
+  </si>
+  <si>
+    <t>42.67</t>
+  </si>
+  <si>
+    <t>6.13</t>
+  </si>
+  <si>
+    <t>40.62</t>
+  </si>
+  <si>
+    <t>7.12</t>
+  </si>
+  <si>
+    <t>38.83</t>
+  </si>
+  <si>
+    <t>8.48</t>
+  </si>
+  <si>
+    <t>37.56</t>
+  </si>
+  <si>
+    <t>10.07</t>
+  </si>
+  <si>
+    <t>36.41</t>
+  </si>
+  <si>
+    <t>FBK-LF W16-S18 1.5e15</t>
+  </si>
+  <si>
+    <t>FBK-LF W16-S25 - 1e15</t>
+  </si>
+  <si>
+    <t>FBK-LF W18-S2 - 1e15</t>
+  </si>
+  <si>
+    <t>1.91</t>
+  </si>
+  <si>
+    <t>81.18</t>
+  </si>
+  <si>
+    <t>2.32</t>
+  </si>
+  <si>
+    <t>74.86</t>
+  </si>
+  <si>
+    <t>2.92</t>
+  </si>
+  <si>
+    <t>57.63</t>
+  </si>
+  <si>
+    <t>3.79</t>
+  </si>
+  <si>
+    <t>51.97</t>
+  </si>
+  <si>
+    <t>4.82</t>
+  </si>
+  <si>
+    <t>46.24</t>
+  </si>
+  <si>
+    <t>5.65</t>
+  </si>
+  <si>
+    <t>43.43</t>
+  </si>
+  <si>
+    <t>6.56</t>
+  </si>
+  <si>
+    <t>41.94</t>
+  </si>
+  <si>
+    <t>7.81</t>
+  </si>
+  <si>
+    <t>40.03</t>
+  </si>
+  <si>
+    <t>9.39</t>
+  </si>
+  <si>
+    <t>39.51</t>
+  </si>
+  <si>
+    <t>FBK-LF W16-S2 1.5e15</t>
   </si>
 </sst>
 </file>
@@ -848,32 +1197,32 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="J2" s="4" t="s">
-        <v>57</v>
+        <v>180</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="N2" s="5" t="s">
-        <v>62</v>
+        <v>181</v>
       </c>
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
       <c r="R2" s="3" t="s">
-        <v>77</v>
+        <v>182</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="V2" s="3" t="s">
-        <v>91</v>
+        <v>183</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Z2" s="3" t="s">
-        <v>106</v>
+        <v>184</v>
       </c>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AD2" s="3" t="s">
-        <v>106</v>
+        <v>184</v>
       </c>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
@@ -993,37 +1342,37 @@
         <v>300</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="V4" s="2">
         <v>300</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="Z4" s="2">
         <v>300</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="AB4" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AD4" s="2">
         <v>300</v>
       </c>
       <c r="AE4" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="AF4" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="2:32" x14ac:dyDescent="0.2">
@@ -1049,7 +1398,7 @@
         <v>250</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>46</v>
@@ -1061,43 +1410,43 @@
         <v>53</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R5" s="2">
         <v>350</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="V5" s="2">
         <v>350</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="Z5" s="2">
         <v>350</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="AD5" s="2">
         <v>350</v>
       </c>
       <c r="AE5" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="AF5" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="2:32" x14ac:dyDescent="0.2">
@@ -1123,7 +1472,7 @@
         <v>300</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>47</v>
@@ -1135,43 +1484,43 @@
         <v>54</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="R6" s="2">
         <v>400</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V6" s="2">
         <v>400</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="Z6" s="2">
         <v>400</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AD6" s="2">
         <v>400</v>
       </c>
       <c r="AE6" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="AF6" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="2:32" x14ac:dyDescent="0.2">
@@ -1197,7 +1546,7 @@
         <v>325</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>48</v>
@@ -1209,43 +1558,43 @@
         <v>55</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="R7" s="2">
         <v>450</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="V7" s="2">
         <v>450</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="X7" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="Z7" s="2">
         <v>450</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="AB7" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="AD7" s="2">
         <v>450</v>
       </c>
       <c r="AE7" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="AF7" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="2:32" x14ac:dyDescent="0.2">
@@ -1271,7 +1620,7 @@
         <v>350</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>49</v>
@@ -1283,43 +1632,43 @@
         <v>56</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="R8" s="2">
         <v>500</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="V8" s="2">
         <v>500</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="Z8" s="2">
         <v>500</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="AD8" s="2">
         <v>500</v>
       </c>
       <c r="AE8" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="AF8" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="2:32" x14ac:dyDescent="0.2">
@@ -1354,37 +1703,37 @@
         <v>525</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="V9" s="2">
         <v>525</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Z9" s="2">
         <v>525</v>
       </c>
       <c r="AA9" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="AB9" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AD9" s="2">
         <v>525</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="AF9" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="2:32" x14ac:dyDescent="0.2">
@@ -1410,7 +1759,7 @@
         <v>375</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>51</v>
@@ -1419,37 +1768,37 @@
         <v>550</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="V10" s="2">
         <v>550</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="Z10" s="2">
         <v>550</v>
       </c>
       <c r="AA10" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="AB10" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="AD10" s="2">
         <v>550</v>
       </c>
       <c r="AE10" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="AF10" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="2:32" x14ac:dyDescent="0.2">
@@ -1525,4 +1874,637 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1EE5E96-18AA-F34C-AA6B-105E9C7B2B68}">
+  <dimension ref="B2:X13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="J2" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="N2" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="R2" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="V2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+    </row>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2">
+        <v>120</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F4" s="2">
+        <v>120</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J4" s="2">
+        <v>300</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="N4" s="2">
+        <v>300</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="R4" s="2">
+        <v>300</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="V4" s="2">
+        <v>300</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B5" s="2">
+        <v>130</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="2">
+        <v>130</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="J5" s="2">
+        <v>350</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N5" s="2">
+        <v>350</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="R5" s="2">
+        <v>350</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="V5" s="2">
+        <v>350</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B6" s="2">
+        <v>140</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="2">
+        <v>140</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J6" s="2">
+        <v>400</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="N6" s="2">
+        <v>400</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="R6" s="2">
+        <v>400</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="V6" s="2">
+        <v>400</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B7" s="2">
+        <v>150</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F7" s="2">
+        <v>150</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="2">
+        <v>450</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="N7" s="2">
+        <v>450</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="R7" s="2">
+        <v>450</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="V7" s="2">
+        <v>450</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B8" s="2">
+        <v>160</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="2">
+        <v>160</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J8" s="2">
+        <v>500</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="N8" s="2">
+        <v>500</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="R8" s="2">
+        <v>500</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="V8" s="2">
+        <v>500</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B9" s="2">
+        <v>170</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="2">
+        <v>170</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="J9" s="2">
+        <v>525</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="N9" s="2">
+        <v>525</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="R9" s="2">
+        <v>525</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="V9" s="2">
+        <v>525</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B10" s="2">
+        <v>180</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F10" s="2">
+        <v>180</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="J10" s="2">
+        <v>550</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="N10" s="2">
+        <v>550</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="R10" s="2">
+        <v>550</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="V10" s="2">
+        <v>550</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B11" s="2">
+        <v>190</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F11" s="2">
+        <v>190</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J11" s="2">
+        <v>575</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="N11" s="2">
+        <v>575</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="R11" s="2">
+        <v>575</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="V11" s="2">
+        <v>575</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B12" s="2">
+        <v>200</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="2">
+        <v>200</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="J12" s="2">
+        <v>600</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="N12" s="2">
+        <v>600</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R12" s="2">
+        <v>600</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="V12" s="2">
+        <v>600</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B13" s="2">
+        <v>210</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F13" s="2">
+        <v>210</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="V2:X2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add third production (FBK-LC1); per-family config lookup; HPK->HPK6 rename
- config: q_inf_for()/v_seb_for() resolve a production by exact name then by family
  (FBK*/HPK*), so new sheets (e.g. FBK-LC1) get the right bulk Q_inf (0.55) and
  V_SEB (605) with no config edits. model/plots use these helpers.
- Workbook now has HPK6, FBK-LF, FBK-LC1; the HPK sheet was renamed HPK6, so the
  simulation overlay file is renamed simulation/HPK6.csv to match.
- FBK-LC1 fits cleanly at 1e15/1.5e15 (RMS 0.6) and converges to ~0.5 fC; the
  global RMS (1.47) is driven by the steep unirradiated (phi=0) curve and the
  ~5 fC sensor-to-sensor spread there, not by the fit.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parametrization_data.xlsx
+++ b/parametrization_data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardolanteri/Desktop/Parametrization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA24018-27EA-6B47-BA82-16323926586C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59699C6F-B3EC-6C4A-86D5-9800C5831880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
   </bookViews>
   <sheets>
-    <sheet name="HPK" sheetId="1" r:id="rId1"/>
+    <sheet name="HPK6" sheetId="1" r:id="rId1"/>
     <sheet name="FBK-LF" sheetId="2" r:id="rId2"/>
+    <sheet name="FBK-LC1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="315">
   <si>
     <t>V</t>
   </si>
@@ -766,13 +767,232 @@
   </si>
   <si>
     <t>FBK-LF W16-S2 1.5e15</t>
+  </si>
+  <si>
+    <t>11.6</t>
+  </si>
+  <si>
+    <t>38.6</t>
+  </si>
+  <si>
+    <t>14.9</t>
+  </si>
+  <si>
+    <t>19.4</t>
+  </si>
+  <si>
+    <t>34.6</t>
+  </si>
+  <si>
+    <t>24.3</t>
+  </si>
+  <si>
+    <t>31.1</t>
+  </si>
+  <si>
+    <t>29.7</t>
+  </si>
+  <si>
+    <t>31.2</t>
+  </si>
+  <si>
+    <t>37.9</t>
+  </si>
+  <si>
+    <t>30.1</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>50.2</t>
+  </si>
+  <si>
+    <t>13.3</t>
+  </si>
+  <si>
+    <t>45.1</t>
+  </si>
+  <si>
+    <t>16.9</t>
+  </si>
+  <si>
+    <t>38.8</t>
+  </si>
+  <si>
+    <t>29.6</t>
+  </si>
+  <si>
+    <t>32.1</t>
+  </si>
+  <si>
+    <t>38.1</t>
+  </si>
+  <si>
+    <t>32.0</t>
+  </si>
+  <si>
+    <t>FBK-LF W1 5-4 A</t>
+  </si>
+  <si>
+    <t>FBK-LF W1 5-4 B</t>
+  </si>
+  <si>
+    <t>3.35</t>
+  </si>
+  <si>
+    <t>62.3</t>
+  </si>
+  <si>
+    <t>4.55</t>
+  </si>
+  <si>
+    <t>50.16</t>
+  </si>
+  <si>
+    <t>6.12</t>
+  </si>
+  <si>
+    <t>41.03</t>
+  </si>
+  <si>
+    <t>8.85</t>
+  </si>
+  <si>
+    <t>37.21</t>
+  </si>
+  <si>
+    <t>14.26</t>
+  </si>
+  <si>
+    <t>34.62</t>
+  </si>
+  <si>
+    <t>20.7</t>
+  </si>
+  <si>
+    <t>33.19</t>
+  </si>
+  <si>
+    <t>21.7</t>
+  </si>
+  <si>
+    <t>35.1</t>
+  </si>
+  <si>
+    <t>FBK-LF W1 S1 - 1e15</t>
+  </si>
+  <si>
+    <t>3.67</t>
+  </si>
+  <si>
+    <t>54.0</t>
+  </si>
+  <si>
+    <t>4.78</t>
+  </si>
+  <si>
+    <t>44.0</t>
+  </si>
+  <si>
+    <t>5.97</t>
+  </si>
+  <si>
+    <t>39.5</t>
+  </si>
+  <si>
+    <t>9.25</t>
+  </si>
+  <si>
+    <t>14.39</t>
+  </si>
+  <si>
+    <t>30.8</t>
+  </si>
+  <si>
+    <t>20.46</t>
+  </si>
+  <si>
+    <t>30.4</t>
+  </si>
+  <si>
+    <t>30.7</t>
+  </si>
+  <si>
+    <t>FBK-LF W1 S2 - 1e15</t>
+  </si>
+  <si>
+    <t>FBK-LF W1 S3 - 1.5e15</t>
+  </si>
+  <si>
+    <t>3.00</t>
+  </si>
+  <si>
+    <t>48.9</t>
+  </si>
+  <si>
+    <t>3.90</t>
+  </si>
+  <si>
+    <t>43.4</t>
+  </si>
+  <si>
+    <t>5.10</t>
+  </si>
+  <si>
+    <t>39.0</t>
+  </si>
+  <si>
+    <t>7.10</t>
+  </si>
+  <si>
+    <t>37.7</t>
+  </si>
+  <si>
+    <t>9.90</t>
+  </si>
+  <si>
+    <t>35.9</t>
+  </si>
+  <si>
+    <t>3.13</t>
+  </si>
+  <si>
+    <t>53.1</t>
+  </si>
+  <si>
+    <t>3.66</t>
+  </si>
+  <si>
+    <t>48.6</t>
+  </si>
+  <si>
+    <t>4.52</t>
+  </si>
+  <si>
+    <t>39.7</t>
+  </si>
+  <si>
+    <t>5.84</t>
+  </si>
+  <si>
+    <t>36.0</t>
+  </si>
+  <si>
+    <t>8.09</t>
+  </si>
+  <si>
+    <t>33.8</t>
+  </si>
+  <si>
+    <t>8.41</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -792,6 +1012,13 @@
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow (Corpo)"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -801,7 +1028,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -824,11 +1051,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -843,6 +1107,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2498,6 +2771,471 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="V2:X2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="R2:T2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2EDE7F6-4144-BC42-897C-74D16D4AFA6C}">
+  <dimension ref="B2:X10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B2" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="J2" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="N2" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="R2" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="S2" s="7"/>
+      <c r="T2" s="8"/>
+      <c r="V2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+    </row>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2">
+        <v>140</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F4" s="2">
+        <v>120</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="J4" s="2">
+        <v>250</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="N4" s="2">
+        <v>250</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="R4" s="2">
+        <v>400</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="V4" s="2">
+        <v>400</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B5" s="2">
+        <v>160</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F5" s="2">
+        <v>140</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="J5" s="2">
+        <v>300</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="N5" s="2">
+        <v>300</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="R5" s="2">
+        <v>450</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="V5" s="2">
+        <v>450</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B6" s="2">
+        <v>180</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F6" s="2">
+        <v>160</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="J6" s="2">
+        <v>350</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="N6" s="2">
+        <v>340</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="R6" s="2">
+        <v>500</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="V6" s="2">
+        <v>500</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B7" s="2">
+        <v>190</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F7" s="2">
+        <v>180</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="J7" s="2">
+        <v>400</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="N7" s="2">
+        <v>400</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="R7" s="2">
+        <v>550</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="V7" s="2">
+        <v>550</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B8" s="2">
+        <v>200</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F8" s="2">
+        <v>190</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="J8" s="2">
+        <v>450</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="N8" s="2">
+        <v>450</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="R8" s="2">
+        <v>600</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="V8" s="2">
+        <v>600</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B9" s="2">
+        <v>210</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F9" s="2">
+        <v>200</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="J9" s="2">
+        <v>500</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="N9" s="2">
+        <v>490</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="V9" s="2">
+        <v>610</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B10" s="2">
+        <v>215</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J10" s="2">
+        <v>510</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="N10" s="2">
+        <v>520</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="J2:L2"/>

</xml_diff>

<commit_message>
Notebook saves all plots; family comparison plots; sim overlay only where available
1) plots.save_all(sensors, results, surfaces) writes the full set of per-production
   plots to Plots/ (overwrite). run.py and a new notebook cell both call it, so
   running the .ipynb now updates Plots/ just like `python run.py --save`.
2) Simulation overlay (charge_bias_*_sim.pdf) is produced ONLY for productions
   that have a simulation/<prod>.csv; LC1 and any future sheet without one get no
   sim plot. _load_sim now matches the CSV by prefix too, so a renamed sheet
   (FBK-LF -> FBK-LF_PreSerie) still finds FBKLF.csv.
3) For each family with >=2 productions, comparison plots: compare_FBK_charge_bias
   (both on the operating-point axes) and compare_FBK_QV (Q(V) per fluence),
   distinct colours per production. charge/bias draws one SEB line/label per
   distinct V_max (no overlap when productions share it).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parametrization_data.xlsx
+++ b/parametrization_data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardolanteri/Desktop/Parametrization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59699C6F-B3EC-6C4A-86D5-9800C5831880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E730C81-B16C-3A42-BB67-D3915E957712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{B65C7759-0474-BA45-8187-5A8BC2A27372}"/>
   </bookViews>
   <sheets>
     <sheet name="HPK6" sheetId="1" r:id="rId1"/>
-    <sheet name="FBK-LF" sheetId="2" r:id="rId2"/>
+    <sheet name="FBK-LF_PreSerie" sheetId="2" r:id="rId2"/>
     <sheet name="FBK-LC1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -1103,12 +1103,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1116,6 +1110,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1469,16 +1469,16 @@
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="7" t="s">
         <v>180</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
       <c r="R2" s="3" t="s">
         <v>182</v>
       </c>
@@ -2811,11 +2811,11 @@
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="S2" s="7"/>
-      <c r="T2" s="8"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="6"/>
       <c r="V2" s="3" t="s">
         <v>241</v>
       </c>
@@ -3236,12 +3236,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="V2:X2"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
-    <mergeCell ref="V2:X2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>